<commit_message>
vault backup: 2026-05-14 16:56:16
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FILES\Projects\MEC202\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8AFAA5E-39D3-40EA-BA3B-8D399D75687B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84E2BA94-D1CB-4FAB-BA66-B751A92A3C85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{4C355368-0098-4D56-92CA-07E48E6BBCFC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>直线轴承</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -175,6 +175,10 @@
   </si>
   <si>
     <t>总价</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PETG哑光黄色</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -247,16 +251,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -596,10 +600,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CE5121F-4F47-4E38-8926-421734493FCF}">
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr defaultRowHeight="17.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="9" style="2"/>
+    <col min="1" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -619,501 +623,502 @@
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4">
         <v>9.75</v>
       </c>
-      <c r="D3" s="1"/>
+      <c r="D3" s="4"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4">
         <v>13.2</v>
       </c>
-      <c r="D4" s="1"/>
+      <c r="D4" s="4"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4">
         <v>3.3</v>
       </c>
-      <c r="D5" s="1"/>
+      <c r="D5" s="4"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="4">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="5">
         <f>C3+C4+C5</f>
         <v>26.25</v>
       </c>
-      <c r="D6" s="4"/>
+      <c r="D6" s="5"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1">
+      <c r="B8" s="4"/>
+      <c r="C8" s="4">
         <v>10.6</v>
       </c>
-      <c r="D8" s="1"/>
+      <c r="D8" s="4"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4">
         <v>10.6</v>
       </c>
-      <c r="D9" s="1"/>
+      <c r="D9" s="4"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="4">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="5">
         <f>C8+C9</f>
         <v>21.2</v>
       </c>
-      <c r="D10" s="4"/>
+      <c r="D10" s="5"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1">
+      <c r="B13" s="4"/>
+      <c r="C13" s="4">
         <v>0.56000000000000005</v>
       </c>
-      <c r="D13" s="1"/>
+      <c r="D13" s="4"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1">
+      <c r="B14" s="4"/>
+      <c r="C14" s="4">
         <v>0.96</v>
       </c>
-      <c r="D14" s="1"/>
+      <c r="D14" s="4"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1">
+      <c r="B15" s="4"/>
+      <c r="C15" s="4">
         <v>1.83</v>
       </c>
-      <c r="D15" s="1"/>
+      <c r="D15" s="4"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1">
+      <c r="B16" s="4"/>
+      <c r="C16" s="4">
         <v>0.83</v>
       </c>
-      <c r="D16" s="1"/>
+      <c r="D16" s="4"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1">
+      <c r="B17" s="4"/>
+      <c r="C17" s="4">
         <v>4.38</v>
       </c>
-      <c r="D17" s="1"/>
+      <c r="D17" s="4"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1">
+      <c r="B18" s="4"/>
+      <c r="C18" s="4">
         <v>1.21</v>
       </c>
-      <c r="D18" s="1"/>
+      <c r="D18" s="4"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1">
+      <c r="B19" s="4"/>
+      <c r="C19" s="4">
         <v>1.97</v>
       </c>
-      <c r="D19" s="1"/>
+      <c r="D19" s="4"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1">
+      <c r="B20" s="4"/>
+      <c r="C20" s="4">
         <v>2.1</v>
       </c>
-      <c r="D20" s="1"/>
+      <c r="D20" s="4"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="4">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="5">
         <f>C13+C14+C15+C16+C17+C18+C19+C20</f>
         <v>13.84</v>
       </c>
-      <c r="D21" s="4"/>
+      <c r="D21" s="5"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="1" t="s">
+      <c r="A23" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="1"/>
-      <c r="C23" s="4">
+      <c r="B23" s="4"/>
+      <c r="C23" s="5">
         <v>6.86</v>
       </c>
-      <c r="D23" s="4"/>
+      <c r="D23" s="5"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B24" s="1"/>
-      <c r="C24" s="4">
+      <c r="B24" s="4"/>
+      <c r="C24" s="5">
         <v>10.9</v>
       </c>
-      <c r="D24" s="4"/>
+      <c r="D24" s="5"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="1"/>
-      <c r="C25" s="4">
+      <c r="B25" s="4"/>
+      <c r="C25" s="5">
         <v>41</v>
       </c>
-      <c r="D25" s="4"/>
+      <c r="D25" s="5"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B26" s="1"/>
-      <c r="C26" s="4">
+      <c r="B26" s="4"/>
+      <c r="C26" s="5">
         <v>8.4</v>
       </c>
-      <c r="D26" s="4"/>
+      <c r="D26" s="5"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="1" t="s">
+      <c r="A28" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="1" t="s">
+      <c r="A29" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1">
+      <c r="B29" s="4"/>
+      <c r="C29" s="4">
         <v>22.9</v>
       </c>
-      <c r="D29" s="1"/>
+      <c r="D29" s="4"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="1" t="s">
+      <c r="A30" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4">
+        <v>22.43</v>
+      </c>
+      <c r="D30" s="4"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B30" s="1"/>
-      <c r="C30" s="1">
+      <c r="B31" s="4"/>
+      <c r="C31" s="4">
         <v>20.9</v>
       </c>
-      <c r="D30" s="1"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="1" t="s">
+      <c r="D31" s="4"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1">
+      <c r="B32" s="4"/>
+      <c r="C32" s="4">
         <v>33.9</v>
       </c>
-      <c r="D31" s="1"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="1"/>
-      <c r="B32" s="1"/>
-      <c r="C32" s="4">
-        <f>C29+C30+C31</f>
-        <v>77.699999999999989</v>
-      </c>
       <c r="D32" s="4"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="1"/>
-      <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
-      <c r="D33" s="1"/>
+      <c r="A33" s="4"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="5">
+        <f>C29+C31+C32+C30</f>
+        <v>100.13</v>
+      </c>
+      <c r="D33" s="5"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="1" t="s">
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B34" s="1"/>
-      <c r="C34" s="4">
+      <c r="B35" s="4"/>
+      <c r="C35" s="5">
         <v>10.119999999999999</v>
       </c>
-      <c r="D34" s="4"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="1"/>
-      <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="1"/>
+      <c r="D35" s="5"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="1" t="s">
+      <c r="A36" s="4"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B36" s="1"/>
-      <c r="C36" s="1"/>
-      <c r="D36" s="1"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="1" t="s">
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B37" s="1"/>
-      <c r="C37" s="1">
+      <c r="B38" s="4"/>
+      <c r="C38" s="4">
         <v>13.37</v>
       </c>
-      <c r="D37" s="1"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="1" t="s">
+      <c r="D38" s="4"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B38" s="1"/>
-      <c r="C38" s="1">
+      <c r="B39" s="4"/>
+      <c r="C39" s="4">
         <v>20.5</v>
       </c>
-      <c r="D38" s="1"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="1"/>
-      <c r="B39" s="1"/>
-      <c r="C39" s="4">
-        <f>C37+C38</f>
+      <c r="D39" s="4"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" s="4"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="5">
+        <f>C38+C39</f>
         <v>33.869999999999997</v>
       </c>
-      <c r="D39" s="4"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="1"/>
-      <c r="B40" s="1"/>
-      <c r="C40" s="1"/>
-      <c r="D40" s="1"/>
+      <c r="D40" s="5"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="1" t="s">
+      <c r="A41" s="4"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B41" s="1"/>
-      <c r="C41" s="4">
+      <c r="B42" s="4"/>
+      <c r="C42" s="5">
         <v>46.6</v>
       </c>
-      <c r="D41" s="4"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="1" t="s">
+      <c r="D42" s="5"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B42" s="1"/>
-      <c r="C42" s="4">
+      <c r="B43" s="4"/>
+      <c r="C43" s="5">
         <v>20.059999999999999</v>
       </c>
-      <c r="D42" s="4"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="1" t="s">
+      <c r="D43" s="5"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B43" s="1"/>
-      <c r="C43" s="4">
+      <c r="B44" s="4"/>
+      <c r="C44" s="5">
         <v>74</v>
       </c>
-      <c r="D43" s="4"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="1" t="s">
+      <c r="D44" s="5"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B44" s="1"/>
-      <c r="C44" s="4">
+      <c r="B45" s="4"/>
+      <c r="C45" s="5">
         <v>1.6</v>
       </c>
-      <c r="D44" s="4"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="1" t="s">
+      <c r="D45" s="5"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B45" s="1"/>
-      <c r="C45" s="4">
+      <c r="B46" s="4"/>
+      <c r="C46" s="5">
         <v>4.01</v>
       </c>
-      <c r="D45" s="4"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="1" t="s">
+      <c r="D46" s="5"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B46" s="1"/>
-      <c r="C46" s="4">
+      <c r="B47" s="4"/>
+      <c r="C47" s="5">
         <v>34.979999999999997</v>
       </c>
-      <c r="D46" s="4"/>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="1" t="s">
+      <c r="D47" s="5"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B47" s="1"/>
-      <c r="C47" s="4">
+      <c r="B48" s="4"/>
+      <c r="C48" s="5">
         <v>12.25</v>
       </c>
-      <c r="D47" s="4"/>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="1" t="s">
+      <c r="D48" s="5"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B48" s="1"/>
-      <c r="C48" s="4">
+      <c r="B49" s="4"/>
+      <c r="C49" s="5">
         <v>60</v>
       </c>
-      <c r="D48" s="4"/>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="1" t="s">
+      <c r="D49" s="5"/>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B49" s="1"/>
-      <c r="C49" s="4">
+      <c r="B50" s="4"/>
+      <c r="C50" s="5">
         <v>38.99</v>
       </c>
-      <c r="D49" s="4"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" s="1"/>
-      <c r="B50" s="1"/>
-      <c r="C50" s="1"/>
-      <c r="D50" s="1"/>
+      <c r="D50" s="5"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" s="3" t="s">
+      <c r="A51" s="4"/>
+      <c r="B51" s="4"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="4"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B51" s="3"/>
-      <c r="C51" s="3">
-        <f>C6+C10+C21+C23+C24+C26++C25+C32+C34+C39+C41+C42+C43+C44+C45+C46+C47+C48+C49</f>
-        <v>542.63</v>
-      </c>
-      <c r="D51" s="3"/>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="3"/>
       <c r="B52" s="3"/>
-      <c r="C52" s="3"/>
+      <c r="C52" s="3">
+        <f>C6+C10+C21+C23+C24+C26++C25+C33+C35+C40+C42+C43+C44+C45+C46+C47+C48+C49+C50</f>
+        <v>565.06000000000006</v>
+      </c>
       <c r="D52" s="3"/>
     </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" s="3"/>
+      <c r="B53" s="3"/>
+      <c r="C53" s="3"/>
+      <c r="D53" s="3"/>
+    </row>
   </sheetData>
-  <mergeCells count="99">
-    <mergeCell ref="A51:B52"/>
-    <mergeCell ref="C51:D52"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A50:B50"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="C48:D48"/>
-    <mergeCell ref="C49:D49"/>
-    <mergeCell ref="C50:D50"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="C31:D31"/>
+  <mergeCells count="101">
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="C26:D26"/>
@@ -1129,46 +1134,58 @@
     <mergeCell ref="C24:D24"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A19:B19"/>
     <mergeCell ref="A21:B21"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="C1:D2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="C49:D49"/>
+    <mergeCell ref="C50:D50"/>
+    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="A52:B53"/>
+    <mergeCell ref="C52:D53"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A51:B51"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>